<commit_message>
añadida plantilla nueva, borrado manual y orden de la tabla
</commit_message>
<xml_diff>
--- a/public/excel/PLANTILLA_ZONA_SUR.xlsx
+++ b/public/excel/PLANTILLA_ZONA_SUR.xlsx
@@ -27,36 +27,59 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
-    <t>fecha</t>
+    <t>FECHA</t>
   </si>
   <si>
-    <t>referencia_del_vehiculo</t>
+    <t>MES</t>
   </si>
   <si>
-    <t>descripcion</t>
+    <t>NºVEHICULO</t>
   </si>
   <si>
-    <t>monto_euro</t>
+    <t>CONCEPTO</t>
   </si>
   <si>
-    <t>PASTILLAS FRENOS TEXTAR</t>
+    <t>CANTIDAD</t>
   </si>
   <si>
-    <t>ITV</t>
+    <t>PRECIO</t>
+  </si>
+  <si>
+    <t>DESCUENTO</t>
+  </si>
+  <si>
+    <t>TOTAL</t>
+  </si>
+  <si>
+    <t>PROVEEDOR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FILTROS </t>
+  </si>
+  <si>
+    <t>GRUPO CARTES</t>
+  </si>
+  <si>
+    <t>TABLERO FENOLICO 2,5X1,23</t>
+  </si>
+  <si>
+    <t>SUMICALL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="5">
+  <numFmts count="7">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="176" formatCode="_-&quot;€&quot;* #,##0.00_-;\-&quot;€&quot;* #,##0.00_-;_-&quot;€&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-* #,##0_-;\-&quot;€&quot;* #,##0_-;_-&quot;€&quot;* &quot;-&quot;_-;_-@_-"/>
-    <numFmt numFmtId="178" formatCode="dd\-mm\-yy;@"/>
+    <numFmt numFmtId="178" formatCode="d\-m;@"/>
+    <numFmt numFmtId="179" formatCode="#,##0.00\ &quot;€&quot;"/>
+    <numFmt numFmtId="180" formatCode="dd\-mm\-yy;@"/>
   </numFmts>
   <fonts count="24">
     <font>
@@ -68,15 +91,17 @@
     <font>
       <b/>
       <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="1"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
@@ -235,12 +260,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="34">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor theme="4"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -435,7 +466,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="11">
+  <borders count="15">
     <border>
       <left/>
       <right/>
@@ -445,16 +476,16 @@
     </border>
     <border>
       <left style="thin">
-        <color auto="1"/>
+        <color theme="4" tint="0.399975585192419"/>
       </left>
       <right style="thin">
-        <color auto="1"/>
+        <color theme="0"/>
       </right>
       <top style="thin">
-        <color auto="1"/>
+        <color theme="4" tint="0.399975585192419"/>
       </top>
       <bottom style="thin">
-        <color auto="1"/>
+        <color theme="0"/>
       </bottom>
       <diagonal/>
     </border>
@@ -464,6 +495,66 @@
       </left>
       <right style="thin">
         <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.399975585192419"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="4" tint="0.399975585192419"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.399975585192419"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.399975585192419"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="4" tint="0.399975585192419"/>
+      </right>
+      <top style="thin">
+        <color theme="4" tint="0.399975585192419"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="4" tint="0.399975585192419"/>
       </right>
       <top style="thin">
         <color theme="0"/>
@@ -585,7 +676,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="3" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -597,139 +688,163 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="10" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="13" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="178" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="178" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="179" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="178" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="180" fontId="2" fillId="3" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="3" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="180" fontId="2" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1186,54 +1301,101 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultColWidth="8.54285714285714" defaultRowHeight="15" outlineLevelRow="2" outlineLevelCol="3"/>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr defaultColWidth="8.54285714285714" defaultRowHeight="15" outlineLevelRow="2"/>
   <cols>
     <col min="2" max="2" width="21.5714285714286" customWidth="1"/>
     <col min="3" max="3" width="31.1428571428571" customWidth="1"/>
     <col min="4" max="4" width="37.2857142857143" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="I1" s="13" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="2">
-        <v>45659</v>
-      </c>
-      <c r="B2" s="3">
-        <v>3132</v>
-      </c>
-      <c r="C2" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" s="4">
-        <v>51.08</v>
+    <row r="2" spans="1:9">
+      <c r="A2" s="5">
+        <v>45293</v>
+      </c>
+      <c r="B2" s="6" t="str">
+        <f>TEXT(A2,"MMMM")</f>
+        <v>enero</v>
+      </c>
+      <c r="C2" s="6">
+        <v>2269</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="6">
+        <v>1</v>
+      </c>
+      <c r="F2" s="7">
+        <v>198.99</v>
+      </c>
+      <c r="G2" s="8"/>
+      <c r="H2" s="7">
+        <f>F2*E2*(1-G2)</f>
+        <v>198.99</v>
+      </c>
+      <c r="I2" s="14" t="s">
+        <v>10</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="5">
-        <v>45659</v>
-      </c>
-      <c r="B3" s="6">
-        <v>3134</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="7">
-        <v>50.87</v>
+    <row r="3" spans="1:9">
+      <c r="A3" s="9">
+        <v>45293</v>
+      </c>
+      <c r="B3" s="10" t="str">
+        <f>TEXT(A3,"MMMM")</f>
+        <v>enero</v>
+      </c>
+      <c r="C3" s="10">
+        <v>3036</v>
+      </c>
+      <c r="D3" s="10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" s="10">
+        <v>12.5</v>
+      </c>
+      <c r="F3" s="11">
+        <v>62.7</v>
+      </c>
+      <c r="G3" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="H3" s="11">
+        <f>F3*E3*(1-G3)</f>
+        <v>587.8125</v>
+      </c>
+      <c r="I3" s="15" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>